<commit_message>
Version actualizada del cehcklist
</commit_message>
<xml_diff>
--- a/Checklist_RF_Completado (2).xlsx
+++ b/Checklist_RF_Completado (2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Veron\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13A277C-05AF-4EB1-9501-653B1AAEEF59}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4619C48-87F4-4104-9FF9-5019786A1D14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
@@ -166,6 +166,12 @@
   </si>
   <si>
     <t>CUMPLE: 3 |  PARCIAL: 9  |  NO CUMPLE: 3  (de 15 RF evaluados)</t>
+  </si>
+  <si>
+    <t>Casos de pruebas</t>
+  </si>
+  <si>
+    <t>SI</t>
   </si>
 </sst>
 </file>
@@ -579,19 +585,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="6" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -614,13 +620,16 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>44</v>
       </c>
@@ -642,14 +651,17 @@
       <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="9" t="s">
+      <c r="H2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -671,14 +683,17 @@
       <c r="G3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="H3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -700,14 +715,17 @@
       <c r="G4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="7" t="s">
+      <c r="H4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -729,14 +747,17 @@
       <c r="G5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="7" t="s">
+      <c r="H5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
@@ -758,14 +779,17 @@
       <c r="G6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -790,11 +814,14 @@
       <c r="H7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
@@ -816,14 +843,17 @@
       <c r="G8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="7" t="s">
+      <c r="H8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>26</v>
       </c>
@@ -845,14 +875,17 @@
       <c r="G9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="8" t="s">
+      <c r="H9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
@@ -877,11 +910,14 @@
       <c r="H10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>31</v>
       </c>
@@ -903,14 +939,17 @@
       <c r="G11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" s="7" t="s">
+      <c r="H11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -932,14 +971,17 @@
       <c r="G12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="7" t="s">
+      <c r="H12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -961,14 +1003,17 @@
       <c r="G13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" s="7" t="s">
+      <c r="H13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>37</v>
       </c>
@@ -990,14 +1035,17 @@
       <c r="G14" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" s="8" t="s">
+      <c r="H14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>39</v>
       </c>
@@ -1019,14 +1067,17 @@
       <c r="G15" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="8" t="s">
+      <c r="H15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>41</v>
       </c>
@@ -1048,14 +1099,17 @@
       <c r="G16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="7" t="s">
+      <c r="H16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>43</v>
       </c>
@@ -1063,7 +1117,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1073,10 +1127,11 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B20:J20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>